<commit_message>
Update jd-Rating Skill output
</commit_message>
<xml_diff>
--- a/skills/jd-rating/assets/JD-Rating-Template.xlsx
+++ b/skills/jd-rating/assets/JD-Rating-Template.xlsx
@@ -224,7 +224,7 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="7" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -301,6 +301,18 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -758,11 +770,11 @@
   <dimension ref="B6:I38"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col width="7.1640625" customWidth="1" min="1" max="1"/>
-    <col width="6" customWidth="1" min="2" max="2"/>
-    <col width="52" customWidth="1" min="3" max="3"/>
+    <col hidden="1" min="1" max="1"/>
+    <col width="4" customWidth="1" min="2" max="2"/>
+    <col width="45" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col hidden="1" width="67.5" customWidth="1" min="5" max="5"/>
+    <col width="55" customWidth="1" min="5" max="5"/>
     <col width="47.1640625" customWidth="1" min="6" max="6"/>
     <col hidden="1" width="23.1640625" customWidth="1" min="9" max="9"/>
   </cols>
@@ -802,7 +814,7 @@
         </is>
       </c>
     </row>
-    <row r="9">
+    <row r="9" ht="16" customHeight="1">
       <c r="B9" s="17" t="inlineStr">
         <is>
           <t>1. Job Title</t>
@@ -828,7 +840,7 @@
         </is>
       </c>
       <c r="D10" s="3" t="n"/>
-      <c r="E10" s="21" t="n"/>
+      <c r="E10" s="28" t="n"/>
       <c r="F10" s="22" t="n"/>
       <c r="I10" t="inlineStr">
         <is>
@@ -847,7 +859,7 @@
         </is>
       </c>
       <c r="D11" s="3" t="n"/>
-      <c r="E11" s="8" t="n"/>
+      <c r="E11" s="29" t="n"/>
       <c r="F11" s="20" t="n"/>
       <c r="I11" t="inlineStr">
         <is>
@@ -855,7 +867,7 @@
         </is>
       </c>
     </row>
-    <row r="12">
+    <row r="12" ht="16" customHeight="1">
       <c r="B12" s="17" t="inlineStr">
         <is>
           <t>2. Job Summary / Overview</t>
@@ -876,7 +888,7 @@
         </is>
       </c>
       <c r="D13" s="3" t="n"/>
-      <c r="E13" s="10" t="n"/>
+      <c r="E13" s="29" t="n"/>
     </row>
     <row r="14" ht="16" customHeight="1">
       <c r="B14" s="25">
@@ -889,7 +901,7 @@
         </is>
       </c>
       <c r="D14" s="3" t="n"/>
-      <c r="E14" s="10" t="n"/>
+      <c r="E14" s="29" t="n"/>
     </row>
     <row r="15" ht="16" customHeight="1">
       <c r="B15" s="25">
@@ -902,7 +914,7 @@
         </is>
       </c>
       <c r="D15" s="3" t="n"/>
-      <c r="E15" s="10" t="n"/>
+      <c r="E15" s="29" t="n"/>
     </row>
     <row r="16" ht="16" customHeight="1">
       <c r="B16" s="26">
@@ -915,7 +927,7 @@
         </is>
       </c>
       <c r="D16" s="3" t="n"/>
-      <c r="E16" s="10" t="n"/>
+      <c r="E16" s="29" t="n"/>
     </row>
     <row r="17" ht="16" customHeight="1">
       <c r="B17" s="26">
@@ -928,9 +940,9 @@
         </is>
       </c>
       <c r="D17" s="3" t="n"/>
-      <c r="E17" s="10" t="n"/>
-    </row>
-    <row r="18">
+      <c r="E17" s="29" t="n"/>
+    </row>
+    <row r="18" ht="16" customHeight="1">
       <c r="B18" s="17" t="inlineStr">
         <is>
           <t>3. Key Responsibilities / Duties</t>
@@ -951,7 +963,7 @@
         </is>
       </c>
       <c r="D19" s="3" t="n"/>
-      <c r="E19" s="8" t="n"/>
+      <c r="E19" s="29" t="n"/>
     </row>
     <row r="20" ht="16" customHeight="1">
       <c r="B20" s="25">
@@ -964,9 +976,9 @@
         </is>
       </c>
       <c r="D20" s="3" t="n"/>
-      <c r="E20" s="10" t="n"/>
-    </row>
-    <row r="21">
+      <c r="E20" s="29" t="n"/>
+    </row>
+    <row r="21" ht="16" customHeight="1">
       <c r="B21" s="17" t="inlineStr">
         <is>
           <t>4. Required Qualifications (Must-Haves)</t>
@@ -987,7 +999,7 @@
         </is>
       </c>
       <c r="D22" s="3" t="n"/>
-      <c r="E22" s="10" t="n"/>
+      <c r="E22" s="29" t="n"/>
     </row>
     <row r="23" ht="16" customHeight="1">
       <c r="B23" s="25">
@@ -1000,7 +1012,7 @@
         </is>
       </c>
       <c r="D23" s="3" t="n"/>
-      <c r="E23" s="10" t="n"/>
+      <c r="E23" s="29" t="n"/>
     </row>
     <row r="24" ht="16" customHeight="1">
       <c r="B24" s="25">
@@ -1013,9 +1025,9 @@
         </is>
       </c>
       <c r="D24" s="3" t="n"/>
-      <c r="E24" s="8" t="n"/>
-    </row>
-    <row r="25">
+      <c r="E24" s="29" t="n"/>
+    </row>
+    <row r="25" ht="16" customHeight="1">
       <c r="B25" s="17" t="inlineStr">
         <is>
           <t>5. Preferred Qualifications (Nice-to-Haves)</t>
@@ -1036,7 +1048,7 @@
         </is>
       </c>
       <c r="D26" s="3" t="n"/>
-      <c r="E26" s="8" t="n"/>
+      <c r="E26" s="29" t="n"/>
     </row>
     <row r="27" ht="16" customHeight="1">
       <c r="B27" s="25">
@@ -1049,7 +1061,7 @@
         </is>
       </c>
       <c r="D27" s="3" t="n"/>
-      <c r="E27" s="10" t="n"/>
+      <c r="E27" s="29" t="n"/>
     </row>
     <row r="28" ht="16" customHeight="1">
       <c r="B28" s="25">
@@ -1062,9 +1074,9 @@
         </is>
       </c>
       <c r="D28" s="3" t="n"/>
-      <c r="E28" s="10" t="n"/>
-    </row>
-    <row r="29">
+      <c r="E28" s="29" t="n"/>
+    </row>
+    <row r="29" ht="16" customHeight="1">
       <c r="B29" s="17" t="inlineStr">
         <is>
           <t>6. Skills &amp; Competencies</t>
@@ -1085,7 +1097,7 @@
         </is>
       </c>
       <c r="D30" s="3" t="n"/>
-      <c r="E30" s="9" t="n"/>
+      <c r="E30" s="30" t="n"/>
     </row>
     <row r="31" ht="16" customHeight="1">
       <c r="B31" s="25">
@@ -1098,9 +1110,9 @@
         </is>
       </c>
       <c r="D31" s="3" t="n"/>
-      <c r="E31" s="8" t="n"/>
-    </row>
-    <row r="32">
+      <c r="E31" s="29" t="n"/>
+    </row>
+    <row r="32" ht="16" customHeight="1">
       <c r="B32" s="17" t="inlineStr">
         <is>
           <t>7. Compensation &amp; Benefits</t>
@@ -1121,7 +1133,7 @@
         </is>
       </c>
       <c r="D33" s="3" t="n"/>
-      <c r="E33" s="10" t="n"/>
+      <c r="E33" s="29" t="n"/>
     </row>
     <row r="34" ht="16" customHeight="1">
       <c r="B34" s="25">
@@ -1134,7 +1146,7 @@
         </is>
       </c>
       <c r="D34" s="3" t="n"/>
-      <c r="E34" s="10" t="n"/>
+      <c r="E34" s="29" t="n"/>
     </row>
     <row r="35" ht="16" customHeight="1">
       <c r="B35" s="25">
@@ -1147,7 +1159,7 @@
         </is>
       </c>
       <c r="D35" s="3" t="n"/>
-      <c r="E35" s="10" t="n"/>
+      <c r="E35" s="29" t="n"/>
     </row>
     <row r="36" ht="16" customHeight="1">
       <c r="B36" s="25">
@@ -1160,9 +1172,9 @@
         </is>
       </c>
       <c r="D36" s="3" t="n"/>
-      <c r="E36" s="10" t="n"/>
-    </row>
-    <row r="37">
+      <c r="E36" s="29" t="n"/>
+    </row>
+    <row r="37" ht="20" customHeight="1">
       <c r="B37" s="14" t="inlineStr">
         <is>
           <t>Total items:</t>
@@ -1173,7 +1185,7 @@
         <f>(COUNTIF(D10:D11,"Completed")+COUNTIF(D13:D17,"Completed")+COUNTIF(D19:D20,"Completed")+COUNTIF(D22:D24,"Completed")+COUNTIF(D26:D28,"Completed")+COUNTIF(D30:D31,"Completed")+COUNTIF(D33:D36,"Completed"))/21</f>
         <v/>
       </c>
-      <c r="E37" s="7" t="inlineStr">
+      <c r="E37" s="31" t="inlineStr">
         <is>
           <t>Not Approved - Reworked</t>
         </is>

</xml_diff>